<commit_message>
some updates to this version
</commit_message>
<xml_diff>
--- a/smartshop/EvidenceBasedAdaptiveUI/reports/01_data_cleaning/categorical_quality_summary.xlsx
+++ b/smartshop/EvidenceBasedAdaptiveUI/reports/01_data_cleaning/categorical_quality_summary.xlsx
@@ -452,7 +452,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>200</v>
+        <v>224</v>
       </c>
       <c r="C2" t="n">
         <v>0</v>
@@ -777,7 +777,7 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C27" t="n">
         <v>0</v>
@@ -1193,10 +1193,10 @@
         </is>
       </c>
       <c r="B59" t="n">
-        <v>129</v>
+        <v>142</v>
       </c>
       <c r="C59" t="n">
-        <v>68</v>
+        <v>79</v>
       </c>
     </row>
     <row r="60">
@@ -1206,10 +1206,10 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>127</v>
+        <v>140</v>
       </c>
       <c r="C60" t="n">
-        <v>70</v>
+        <v>81</v>
       </c>
     </row>
   </sheetData>

</xml_diff>